<commit_message>
Rename roster templates and update student upload schema
</commit_message>
<xml_diff>
--- a/assets/templates/Staff Database.xlsx
+++ b/assets/templates/Staff Database.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Staff Database" sheetId="1" r:id="R4ec7619dcf1949db"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="2" r:id="Reba077c76da8426d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Staff Database" sheetId="1" r:id="Reffaa8157f954a53"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="2" r:id="R65b867d109b54522"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -341,16 +341,16 @@
         <x:v>AAIS-T-002</x:v>
       </x:c>
       <x:c r="B3" s="8" t="str">
-        <x:v>Sample Coordinator</x:v>
+        <x:v>Sample Staff</x:v>
       </x:c>
       <x:c r="C3" s="8" t="str">
-        <x:v>coordinator@example.com</x:v>
+        <x:v>staff@example.com</x:v>
       </x:c>
       <x:c r="D3" s="8" t="str">
-        <x:v>pl_teacher</x:v>
+        <x:v>teacher</x:v>
       </x:c>
       <x:c r="E3" s="8" t="str">
-        <x:v>PL Coordinator</x:v>
+        <x:v>Activity Coordinator</x:v>
       </x:c>
       <x:c r="F3" s="8" t="str">
         <x:v>No</x:v>
@@ -561,7 +561,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="15" t="str">
-        <x:v>Required fields: employee_id, name, email, role, campus, grades. designation is optional and may be left blank. Use Yes/No for is_hrt and comma-separated grades.</x:v>
+        <x:v>Required fields: employee_id, name, email, role, campus, grades. designation is optional and may be left blank. Use teacher as the staff role unless Yarra adds more approved roles later. Use Yes/No for is_hrt and comma-separated grades.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>